<commit_message>
Calculated granulometry and source carbon values
</commit_message>
<xml_diff>
--- a/Carbon/d13C_Kelp.xlsx
+++ b/Carbon/d13C_Kelp.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lukaseamus/Desktop/PhD/Papers/Burial/kelp-burial/Carbon/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BD44600-0D37-EF44-95CB-EA8B025543D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6B261B8-D6A0-EA4D-8CF6-21DAE0A2D891}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="18960" yWindow="500" windowWidth="15000" windowHeight="19020" xr2:uid="{D120C0EF-290F-244A-AE4B-CB2F7CD281C3}"/>
   </bookViews>
@@ -62,157 +62,157 @@
     <t>E_1_10_final</t>
   </si>
   <si>
+    <t>Species</t>
+  </si>
+  <si>
+    <t>Ecklonia radiata</t>
+  </si>
+  <si>
+    <t>E_1_preliminary</t>
+  </si>
+  <si>
+    <t>E_2_preliminary</t>
+  </si>
+  <si>
+    <t>E_3_preliminary</t>
+  </si>
+  <si>
+    <t>NA</t>
+  </si>
+  <si>
+    <t>Saccharina latissima</t>
+  </si>
+  <si>
+    <t>S_initial</t>
+  </si>
+  <si>
+    <t>S_1_final</t>
+  </si>
+  <si>
+    <t>S_2_final</t>
+  </si>
+  <si>
+    <t>S_3_final</t>
+  </si>
+  <si>
+    <t>Mass</t>
+  </si>
+  <si>
+    <t>E_1</t>
+  </si>
+  <si>
+    <t>E_2</t>
+  </si>
+  <si>
+    <t>E_3</t>
+  </si>
+  <si>
+    <t>E_4</t>
+  </si>
+  <si>
+    <t>E_5</t>
+  </si>
+  <si>
+    <t>E_6</t>
+  </si>
+  <si>
+    <t>E_7</t>
+  </si>
+  <si>
+    <t>E_8</t>
+  </si>
+  <si>
+    <t>E_9</t>
+  </si>
+  <si>
+    <t>E_10</t>
+  </si>
+  <si>
+    <t>L_H_1</t>
+  </si>
+  <si>
+    <t>L_H_2</t>
+  </si>
+  <si>
+    <t>L_H_3</t>
+  </si>
+  <si>
+    <t>L_H_4</t>
+  </si>
+  <si>
+    <t>L_H_5</t>
+  </si>
+  <si>
+    <t>L_H_6</t>
+  </si>
+  <si>
+    <t>L_H_7</t>
+  </si>
+  <si>
+    <t>L_H_8</t>
+  </si>
+  <si>
+    <t>L_H_9</t>
+  </si>
+  <si>
+    <t>L_H_10</t>
+  </si>
+  <si>
+    <t>L_O_1</t>
+  </si>
+  <si>
+    <t>L_O_2</t>
+  </si>
+  <si>
+    <t>L_O_3</t>
+  </si>
+  <si>
+    <t>L_O_4</t>
+  </si>
+  <si>
+    <t>L_O_5</t>
+  </si>
+  <si>
+    <t>L_O_6</t>
+  </si>
+  <si>
+    <t>L_O_7</t>
+  </si>
+  <si>
+    <t>L_O_8</t>
+  </si>
+  <si>
+    <t>L_O_9</t>
+  </si>
+  <si>
+    <t>L_O_10</t>
+  </si>
+  <si>
+    <t>Laminaria hyperborea</t>
+  </si>
+  <si>
+    <t>Laminaria ochroleuca</t>
+  </si>
+  <si>
+    <t>Standards</t>
+  </si>
+  <si>
+    <t>NBS22, IAEA603, USGS24, USGS41, USGS40</t>
+  </si>
+  <si>
+    <t>Date</t>
+  </si>
+  <si>
+    <t>28.07.22</t>
+  </si>
+  <si>
+    <t>10.04.24</t>
+  </si>
+  <si>
+    <t>26.09.25</t>
+  </si>
+  <si>
     <t>C</t>
-  </si>
-  <si>
-    <t>Species</t>
-  </si>
-  <si>
-    <t>Ecklonia radiata</t>
-  </si>
-  <si>
-    <t>E_1_preliminary</t>
-  </si>
-  <si>
-    <t>E_2_preliminary</t>
-  </si>
-  <si>
-    <t>E_3_preliminary</t>
-  </si>
-  <si>
-    <t>NA</t>
-  </si>
-  <si>
-    <t>Saccharina latissima</t>
-  </si>
-  <si>
-    <t>S_initial</t>
-  </si>
-  <si>
-    <t>S_1_final</t>
-  </si>
-  <si>
-    <t>S_2_final</t>
-  </si>
-  <si>
-    <t>S_3_final</t>
-  </si>
-  <si>
-    <t>Mass</t>
-  </si>
-  <si>
-    <t>E_1</t>
-  </si>
-  <si>
-    <t>E_2</t>
-  </si>
-  <si>
-    <t>E_3</t>
-  </si>
-  <si>
-    <t>E_4</t>
-  </si>
-  <si>
-    <t>E_5</t>
-  </si>
-  <si>
-    <t>E_6</t>
-  </si>
-  <si>
-    <t>E_7</t>
-  </si>
-  <si>
-    <t>E_8</t>
-  </si>
-  <si>
-    <t>E_9</t>
-  </si>
-  <si>
-    <t>E_10</t>
-  </si>
-  <si>
-    <t>L_H_1</t>
-  </si>
-  <si>
-    <t>L_H_2</t>
-  </si>
-  <si>
-    <t>L_H_3</t>
-  </si>
-  <si>
-    <t>L_H_4</t>
-  </si>
-  <si>
-    <t>L_H_5</t>
-  </si>
-  <si>
-    <t>L_H_6</t>
-  </si>
-  <si>
-    <t>L_H_7</t>
-  </si>
-  <si>
-    <t>L_H_8</t>
-  </si>
-  <si>
-    <t>L_H_9</t>
-  </si>
-  <si>
-    <t>L_H_10</t>
-  </si>
-  <si>
-    <t>L_O_1</t>
-  </si>
-  <si>
-    <t>L_O_2</t>
-  </si>
-  <si>
-    <t>L_O_3</t>
-  </si>
-  <si>
-    <t>L_O_4</t>
-  </si>
-  <si>
-    <t>L_O_5</t>
-  </si>
-  <si>
-    <t>L_O_6</t>
-  </si>
-  <si>
-    <t>L_O_7</t>
-  </si>
-  <si>
-    <t>L_O_8</t>
-  </si>
-  <si>
-    <t>L_O_9</t>
-  </si>
-  <si>
-    <t>L_O_10</t>
-  </si>
-  <si>
-    <t>Laminaria hyperborea</t>
-  </si>
-  <si>
-    <t>Laminaria ochroleuca</t>
-  </si>
-  <si>
-    <t>Standards</t>
-  </si>
-  <si>
-    <t>NBS22, IAEA603, USGS24, USGS41, USGS40</t>
-  </si>
-  <si>
-    <t>Date</t>
-  </si>
-  <si>
-    <t>28.07.22</t>
-  </si>
-  <si>
-    <t>10.04.24</t>
-  </si>
-  <si>
-    <t>26.09.25</t>
   </si>
 </sst>
 </file>
@@ -595,39 +595,39 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
       </c>
       <c r="C1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E1" t="s">
-        <v>8</v>
+        <v>58</v>
       </c>
       <c r="F1" t="s">
         <v>1</v>
       </c>
       <c r="G1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B2" t="s">
         <v>3</v>
       </c>
       <c r="C2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E2">
         <v>27.9540816143613</v>
@@ -636,21 +636,21 @@
         <v>-20.596953212341035</v>
       </c>
       <c r="G2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B3" t="s">
         <v>2</v>
       </c>
       <c r="C3" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E3">
         <v>26.953163215155399</v>
@@ -659,21 +659,21 @@
         <v>-20.754585277020318</v>
       </c>
       <c r="G3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B4" t="s">
         <v>4</v>
       </c>
       <c r="C4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E4">
         <v>27.844204597150899</v>
@@ -682,21 +682,21 @@
         <v>-21.602328171376801</v>
       </c>
       <c r="G4" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B5" t="s">
         <v>5</v>
       </c>
       <c r="C5" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E5">
         <v>27.3048979887276</v>
@@ -705,21 +705,21 @@
         <v>153.6816112873135</v>
       </c>
       <c r="G5" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B6" t="s">
         <v>6</v>
       </c>
       <c r="C6" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D6" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E6">
         <v>28.7054061514404</v>
@@ -728,21 +728,21 @@
         <v>113.89232989971711</v>
       </c>
       <c r="G6" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B7" t="s">
         <v>7</v>
       </c>
       <c r="C7" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D7" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E7">
         <v>28.603173509199902</v>
@@ -751,87 +751,87 @@
         <v>117.5327505028776</v>
       </c>
       <c r="G7" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B8" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C8" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D8" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E8" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F8">
         <v>626.6410184812803</v>
       </c>
       <c r="G8" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B9" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C9" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D9" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E9" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F9">
         <v>598.67370040362823</v>
       </c>
       <c r="G9" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B10" t="s">
+        <v>12</v>
+      </c>
+      <c r="C10" t="s">
+        <v>9</v>
+      </c>
+      <c r="D10" t="s">
         <v>13</v>
       </c>
-      <c r="C10" t="s">
-        <v>10</v>
-      </c>
-      <c r="D10" t="s">
-        <v>14</v>
-      </c>
       <c r="E10" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F10">
         <v>456.56210283452731</v>
       </c>
       <c r="G10" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B11" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C11" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D11">
         <v>0.53900000000000003</v>
@@ -843,18 +843,18 @@
         <v>-15.263662359636291</v>
       </c>
       <c r="G11" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B12" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C12" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D12">
         <v>0.59</v>
@@ -866,18 +866,18 @@
         <v>165.87149535210742</v>
       </c>
       <c r="G12" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B13" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C13" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D13">
         <v>0.59699999999999998</v>
@@ -889,18 +889,18 @@
         <v>203.81538047418766</v>
       </c>
       <c r="G13" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B14" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C14" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D14">
         <v>0.58399999999999996</v>
@@ -912,18 +912,18 @@
         <v>265.96640930657611</v>
       </c>
       <c r="G14" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B15" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C15" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D15">
         <v>0.55500000000000005</v>
@@ -935,18 +935,18 @@
         <v>492.89302855909921</v>
       </c>
       <c r="G15" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B16" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C16" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D16">
         <v>0.58499999999999996</v>
@@ -958,18 +958,18 @@
         <v>518.45918093005878</v>
       </c>
       <c r="G16" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B17" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C17" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D17">
         <v>0.57299999999999995</v>
@@ -981,18 +981,18 @@
         <v>436.06515266234146</v>
       </c>
       <c r="G17" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B18" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C18" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D18">
         <v>0.58199999999999996</v>
@@ -1004,18 +1004,18 @@
         <v>618.20075294961202</v>
       </c>
       <c r="G18" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B19" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C19" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D19">
         <v>0.54600000000000004</v>
@@ -1027,18 +1027,18 @@
         <v>657.32723962786895</v>
       </c>
       <c r="G19" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B20" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C20" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D20">
         <v>0.59099999999999997</v>
@@ -1050,18 +1050,18 @@
         <v>717.61448572463871</v>
       </c>
       <c r="G20" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B21" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C21" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D21">
         <v>0.54400000000000004</v>
@@ -1073,18 +1073,18 @@
         <v>630.48928798822647</v>
       </c>
       <c r="G21" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B22" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C22" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D22">
         <v>0.56599999999999995</v>
@@ -1096,18 +1096,18 @@
         <v>739.10311347811785</v>
       </c>
       <c r="G22" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B23" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C23" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D23">
         <v>0.51200000000000001</v>
@@ -1119,18 +1119,18 @@
         <v>665.39246280177758</v>
       </c>
       <c r="G23" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B24" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C24" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D24">
         <v>0.51</v>
@@ -1142,18 +1142,18 @@
         <v>755.22879800796397</v>
       </c>
       <c r="G24" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B25" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C25" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D25">
         <v>0.52300000000000002</v>
@@ -1165,18 +1165,18 @@
         <v>443.14799752273007</v>
       </c>
       <c r="G25" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B26" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C26" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D26">
         <v>0.53900000000000003</v>
@@ -1188,18 +1188,18 @@
         <v>515.02190336274282</v>
       </c>
       <c r="G26" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B27" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C27" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D27">
         <v>0.55900000000000005</v>
@@ -1211,18 +1211,18 @@
         <v>493.40225399339715</v>
       </c>
       <c r="G27" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B28" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C28" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D28">
         <v>0.54800000000000004</v>
@@ -1234,18 +1234,18 @@
         <v>460.53602486160912</v>
       </c>
       <c r="G28" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B29" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C29" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D29">
         <v>0.52600000000000002</v>
@@ -1257,18 +1257,18 @@
         <v>468.97307676861385</v>
       </c>
       <c r="G29" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B30" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C30" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D30">
         <v>0.501</v>
@@ -1280,18 +1280,18 @@
         <v>418.63464149040658</v>
       </c>
       <c r="G30" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B31" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C31" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D31">
         <v>0.56399999999999995</v>
@@ -1303,18 +1303,18 @@
         <v>400.57805507899729</v>
       </c>
       <c r="G31" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B32" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C32" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D32">
         <v>0.51300000000000001</v>
@@ -1326,18 +1326,18 @@
         <v>466.98032765189555</v>
       </c>
       <c r="G32" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B33" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C33" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D33">
         <v>0.58699999999999997</v>
@@ -1349,18 +1349,18 @@
         <v>498.45333061330473</v>
       </c>
       <c r="G33" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B34" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C34" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D34">
         <v>0.50700000000000001</v>
@@ -1372,18 +1372,18 @@
         <v>393.74436982075918</v>
       </c>
       <c r="G34" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B35" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C35" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D35">
         <v>0.58299999999999996</v>
@@ -1395,18 +1395,18 @@
         <v>1398.839555036885</v>
       </c>
       <c r="G35" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B36" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C36" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D36">
         <v>0.50600000000000001</v>
@@ -1418,18 +1418,18 @@
         <v>1343.9669419608686</v>
       </c>
       <c r="G36" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B37" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C37" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D37">
         <v>0.52800000000000002</v>
@@ -1441,18 +1441,18 @@
         <v>1414.5375580612422</v>
       </c>
       <c r="G37" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B38" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C38" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D38">
         <v>0.58599999999999997</v>
@@ -1464,18 +1464,18 @@
         <v>1381.1727186136782</v>
       </c>
       <c r="G38" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B39" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C39" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D39">
         <v>0.52200000000000002</v>
@@ -1487,18 +1487,18 @@
         <v>1420.7756493826489</v>
       </c>
       <c r="G39" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B40" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C40" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D40">
         <v>0.52400000000000002</v>
@@ -1510,18 +1510,18 @@
         <v>1262.5742543136532</v>
       </c>
       <c r="G40" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B41" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C41" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D41">
         <v>0.59399999999999997</v>
@@ -1533,18 +1533,18 @@
         <v>1485.6030390113942</v>
       </c>
       <c r="G41" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B42" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C42" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D42">
         <v>0.53</v>
@@ -1556,18 +1556,18 @@
         <v>1269.7488487237897</v>
       </c>
       <c r="G42" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B43" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C43" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D43">
         <v>0.53100000000000003</v>
@@ -1579,18 +1579,18 @@
         <v>1466.2629327656757</v>
       </c>
       <c r="G43" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B44" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C44" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D44">
         <v>0.52</v>
@@ -1602,7 +1602,7 @@
         <v>1331.2600440130552</v>
       </c>
       <c r="G44" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
   </sheetData>

</xml_diff>